<commit_message>
UPDATED env\* : resolved the bugs for the single project single duration
</commit_message>
<xml_diff>
--- a/src/test/env_test_configs/test_configs_matrix.xlsx
+++ b/src/test/env_test_configs/test_configs_matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Career\00. Univesity\Masters\05. Master's thesis\PPO-project-portfolio-budgeting-AI-agent\src\test\env_test_configs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3EC4EF5-D930-4B9B-8B9E-22B6FFD64242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EEF2EEC-1ADE-4C20-969E-8010DC3C97EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -802,13 +802,13 @@
     <t>[[0.3, 0.6, 1.0],[0.3, 0.6, 1.0],[0.3, 0.6, 1.0]]</t>
   </si>
   <si>
-    <t>[2, 3, 4]</t>
-  </si>
-  <si>
-    <t>[[2, 3, 4],[2, 3, 4]]</t>
-  </si>
-  <si>
-    <t>[[2, 3, 4],[2, 3, 4],[2, 3, 4]]</t>
+    <t>[1, 2, 3]</t>
+  </si>
+  <si>
+    <t>[[1, 2, 3],[1, 2, 3]]</t>
+  </si>
+  <si>
+    <t>[[1, 2, 3],[1, 2, 3],[1, 2, 3]]</t>
   </si>
 </sst>
 </file>
@@ -1927,7 +1927,7 @@
         <v>114</v>
       </c>
       <c r="AI3" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ3" s="6"/>
       <c r="AK3" s="6"/>
@@ -2053,7 +2053,7 @@
         <v>114</v>
       </c>
       <c r="DA3" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DB3" s="6"/>
       <c r="DC3" s="6"/>
@@ -2127,7 +2127,7 @@
         <v>114</v>
       </c>
       <c r="AI4" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AJ4" s="6"/>
       <c r="AK4" s="6"/>
@@ -2253,7 +2253,7 @@
         <v>114</v>
       </c>
       <c r="DA4" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DB4" s="6"/>
       <c r="DC4" s="6"/>
@@ -2327,7 +2327,7 @@
         <v>114</v>
       </c>
       <c r="AI5" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AJ5" s="6"/>
       <c r="AK5" s="6"/>
@@ -2527,7 +2527,7 @@
         <v>114</v>
       </c>
       <c r="AI6" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ6" s="6"/>
       <c r="AK6" s="6"/>
@@ -2653,7 +2653,7 @@
         <v>114</v>
       </c>
       <c r="DA6" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DB6" s="6"/>
       <c r="DC6" s="6"/>
@@ -2727,7 +2727,7 @@
         <v>114</v>
       </c>
       <c r="AI7" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AJ7" s="6"/>
       <c r="AK7" s="6"/>
@@ -2927,7 +2927,7 @@
         <v>114</v>
       </c>
       <c r="AI8" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AJ8" s="6"/>
       <c r="AK8" s="6"/>
@@ -3127,9 +3127,9 @@
         <v>114</v>
       </c>
       <c r="AI9" s="8">
-        <v>1</v>
-      </c>
-      <c r="AJ9" s="8"/>
+        <v>0</v>
+      </c>
+      <c r="AJ9" s="6"/>
       <c r="AK9" s="8"/>
       <c r="AL9" s="8"/>
       <c r="AM9" s="8" t="s">
@@ -3253,7 +3253,7 @@
         <v>114</v>
       </c>
       <c r="DA9" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DB9" s="8"/>
       <c r="DC9" s="8"/>
@@ -3327,9 +3327,9 @@
         <v>114</v>
       </c>
       <c r="AI10" s="8">
-        <v>4</v>
-      </c>
-      <c r="AJ10" s="8"/>
+        <v>3</v>
+      </c>
+      <c r="AJ10" s="6"/>
       <c r="AK10" s="8"/>
       <c r="AL10" s="8"/>
       <c r="AM10" s="8" t="s">
@@ -3453,7 +3453,7 @@
         <v>114</v>
       </c>
       <c r="DA10" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DB10" s="8"/>
       <c r="DC10" s="8"/>
@@ -3527,9 +3527,9 @@
         <v>114</v>
       </c>
       <c r="AI11" s="8">
-        <v>4</v>
-      </c>
-      <c r="AJ11" s="8"/>
+        <v>3</v>
+      </c>
+      <c r="AJ11" s="6"/>
       <c r="AK11" s="8"/>
       <c r="AL11" s="8"/>
       <c r="AM11" s="8" t="s">
@@ -3727,9 +3727,9 @@
         <v>114</v>
       </c>
       <c r="AI12" s="8">
-        <v>1</v>
-      </c>
-      <c r="AJ12" s="8"/>
+        <v>0</v>
+      </c>
+      <c r="AJ12" s="6"/>
       <c r="AK12" s="8"/>
       <c r="AL12" s="8"/>
       <c r="AM12" s="8" t="s">
@@ -3853,7 +3853,7 @@
         <v>114</v>
       </c>
       <c r="DA12" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DB12" s="8"/>
       <c r="DC12" s="8"/>
@@ -3927,9 +3927,9 @@
         <v>114</v>
       </c>
       <c r="AI13" s="8">
-        <v>4</v>
-      </c>
-      <c r="AJ13" s="8"/>
+        <v>3</v>
+      </c>
+      <c r="AJ13" s="6"/>
       <c r="AK13" s="8"/>
       <c r="AL13" s="8"/>
       <c r="AM13" s="8" t="s">
@@ -4053,7 +4053,7 @@
         <v>114</v>
       </c>
       <c r="DA13" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DB13" s="8"/>
       <c r="DC13" s="8"/>
@@ -4127,9 +4127,9 @@
         <v>114</v>
       </c>
       <c r="AI14" s="8">
-        <v>4</v>
-      </c>
-      <c r="AJ14" s="8"/>
+        <v>3</v>
+      </c>
+      <c r="AJ14" s="6"/>
       <c r="AK14" s="8"/>
       <c r="AL14" s="8"/>
       <c r="AM14" s="8" t="s">
@@ -4327,9 +4327,9 @@
         <v>114</v>
       </c>
       <c r="AI15" s="8">
-        <v>1</v>
-      </c>
-      <c r="AJ15" s="8"/>
+        <v>0</v>
+      </c>
+      <c r="AJ15" s="6"/>
       <c r="AK15" s="8"/>
       <c r="AL15" s="8"/>
       <c r="AM15" s="8" t="s">
@@ -4453,7 +4453,7 @@
         <v>114</v>
       </c>
       <c r="DA15" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DB15" s="8"/>
       <c r="DC15" s="8"/>
@@ -4527,9 +4527,9 @@
         <v>114</v>
       </c>
       <c r="AI16" s="8">
-        <v>4</v>
-      </c>
-      <c r="AJ16" s="8"/>
+        <v>3</v>
+      </c>
+      <c r="AJ16" s="6"/>
       <c r="AK16" s="8"/>
       <c r="AL16" s="8"/>
       <c r="AM16" s="8" t="s">
@@ -4653,7 +4653,7 @@
         <v>114</v>
       </c>
       <c r="DA16" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DB16" s="8"/>
       <c r="DC16" s="8"/>
@@ -4727,9 +4727,9 @@
         <v>114</v>
       </c>
       <c r="AI17" s="8">
-        <v>4</v>
-      </c>
-      <c r="AJ17" s="8"/>
+        <v>3</v>
+      </c>
+      <c r="AJ17" s="6"/>
       <c r="AK17" s="8"/>
       <c r="AL17" s="8"/>
       <c r="AM17" s="8" t="s">
@@ -4927,9 +4927,9 @@
         <v>114</v>
       </c>
       <c r="AI18" s="11">
-        <v>1</v>
-      </c>
-      <c r="AJ18" s="11"/>
+        <v>0</v>
+      </c>
+      <c r="AJ18" s="6"/>
       <c r="AK18" s="11"/>
       <c r="AL18" s="11"/>
       <c r="AM18" s="11" t="s">
@@ -5053,7 +5053,7 @@
         <v>114</v>
       </c>
       <c r="DA18" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DB18" s="11"/>
       <c r="DC18" s="11"/>
@@ -5127,9 +5127,9 @@
         <v>114</v>
       </c>
       <c r="AI19" s="11">
-        <v>4</v>
-      </c>
-      <c r="AJ19" s="11"/>
+        <v>3</v>
+      </c>
+      <c r="AJ19" s="6"/>
       <c r="AK19" s="11"/>
       <c r="AL19" s="11"/>
       <c r="AM19" s="11" t="s">
@@ -5253,7 +5253,7 @@
         <v>114</v>
       </c>
       <c r="DA19" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DB19" s="11"/>
       <c r="DC19" s="11"/>
@@ -5327,9 +5327,9 @@
         <v>114</v>
       </c>
       <c r="AI20" s="11">
-        <v>4</v>
-      </c>
-      <c r="AJ20" s="11"/>
+        <v>3</v>
+      </c>
+      <c r="AJ20" s="6"/>
       <c r="AK20" s="11"/>
       <c r="AL20" s="11"/>
       <c r="AM20" s="11" t="s">
@@ -5527,9 +5527,9 @@
         <v>114</v>
       </c>
       <c r="AI21" s="11">
-        <v>1</v>
-      </c>
-      <c r="AJ21" s="11"/>
+        <v>0</v>
+      </c>
+      <c r="AJ21" s="6"/>
       <c r="AK21" s="11"/>
       <c r="AL21" s="11"/>
       <c r="AM21" s="11" t="s">
@@ -5653,7 +5653,7 @@
         <v>114</v>
       </c>
       <c r="DA21" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DB21" s="11"/>
       <c r="DC21" s="11"/>
@@ -5727,9 +5727,9 @@
         <v>114</v>
       </c>
       <c r="AI22" s="11">
-        <v>4</v>
-      </c>
-      <c r="AJ22" s="11"/>
+        <v>3</v>
+      </c>
+      <c r="AJ22" s="6"/>
       <c r="AK22" s="11"/>
       <c r="AL22" s="11"/>
       <c r="AM22" s="11" t="s">
@@ -5853,7 +5853,7 @@
         <v>114</v>
       </c>
       <c r="DA22" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DB22" s="11"/>
       <c r="DC22" s="11"/>
@@ -5927,9 +5927,9 @@
         <v>114</v>
       </c>
       <c r="AI23" s="11">
-        <v>4</v>
-      </c>
-      <c r="AJ23" s="11"/>
+        <v>3</v>
+      </c>
+      <c r="AJ23" s="6"/>
       <c r="AK23" s="11"/>
       <c r="AL23" s="11"/>
       <c r="AM23" s="11" t="s">
@@ -6127,9 +6127,9 @@
         <v>114</v>
       </c>
       <c r="AI24" s="11">
-        <v>1</v>
-      </c>
-      <c r="AJ24" s="11"/>
+        <v>0</v>
+      </c>
+      <c r="AJ24" s="6"/>
       <c r="AK24" s="11"/>
       <c r="AL24" s="11"/>
       <c r="AM24" s="11" t="s">
@@ -6253,7 +6253,7 @@
         <v>114</v>
       </c>
       <c r="DA24" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DB24" s="11"/>
       <c r="DC24" s="11"/>
@@ -6327,9 +6327,9 @@
         <v>114</v>
       </c>
       <c r="AI25" s="11">
-        <v>4</v>
-      </c>
-      <c r="AJ25" s="11"/>
+        <v>3</v>
+      </c>
+      <c r="AJ25" s="6"/>
       <c r="AK25" s="11"/>
       <c r="AL25" s="11"/>
       <c r="AM25" s="11" t="s">
@@ -6453,7 +6453,7 @@
         <v>114</v>
       </c>
       <c r="DA25" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DB25" s="11"/>
       <c r="DC25" s="11"/>
@@ -6527,9 +6527,9 @@
         <v>114</v>
       </c>
       <c r="AI26" s="11">
-        <v>4</v>
-      </c>
-      <c r="AJ26" s="11"/>
+        <v>3</v>
+      </c>
+      <c r="AJ26" s="6"/>
       <c r="AK26" s="11"/>
       <c r="AL26" s="11"/>
       <c r="AM26" s="11" t="s">

</xml_diff>